<commit_message>
Add test cases excel file only
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Assignment_1_Test_Automation (2)\Assignment_1_Test_Automation\test_automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT23615120\Assignment_1_Test_Automation\test_automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EB509B9-69EF-4EE3-867F-35E3A3259508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_5BB9D33251298B940D4E53673FB4C93756594B98" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="266">
   <si>
     <t>TC ID</t>
   </si>
@@ -803,15 +803,6 @@
   </si>
   <si>
     <t>Bro, මට කියන්නා තියෙනවා මොනාවද වෙන්නේද කියලා. මම 2025-12-01 වාලාට UK visa apply කරන්නා හිතාගෙනා ඉන්නවා. Appointment එකා 10:30AM වාලාට. Processing fee USD 120 වාගේ තියෙනවා. මේකා හරියනවාද කියලා මට official website එකාට ගිහිල්ලා check කරාගන්නා බෑ, website එකා crash වේලා. කරුණාකරලා ඔයා check කරපු https://gov.uk/visas වාලාට ගිහිල්ලා බලාගන්නා.</t>
-  </si>
-  <si>
-    <t>ERROR: Locator.type: Timeout 30000ms exceeded.
-Call log:
-  - waiting for locator("textarea").first
-    - lo</t>
-  </si>
-  <si>
-    <t>ERROR</t>
   </si>
   <si>
     <t>Rationale: '2025-12-01' is a date format embedded in the Singlish input</t>
@@ -2530,17 +2521,14 @@
       <c r="D77" t="s">
         <v>260</v>
       </c>
-      <c r="E77" t="s">
-        <v>261</v>
-      </c>
       <c r="F77" t="s">
-        <v>262</v>
+        <v>12</v>
       </c>
       <c r="G77" t="s">
         <v>205</v>
       </c>
       <c r="H77" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2548,7 +2536,7 @@
         <v>195</v>
       </c>
       <c r="H78" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="79" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2556,7 +2544,7 @@
         <v>181</v>
       </c>
       <c r="H79" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2564,7 +2552,7 @@
         <v>234</v>
       </c>
       <c r="H80" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="81" spans="7:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2572,7 +2560,7 @@
         <v>117</v>
       </c>
       <c r="H81" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>